<commit_message>
Add first product list data and equivalent
</commit_message>
<xml_diff>
--- a/data/products_list_iter_1.xlsx
+++ b/data/products_list_iter_1.xlsx
@@ -1,316 +1,294 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\SNU Project\agentic-commerce\data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="Calc"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23016" windowHeight="9048" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil1" sheetId="4" r:id="rId1"/>
-    <sheet name="Feuil2" sheetId="5" r:id="rId2"/>
+    <sheet name="Feuil1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Feuil2" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
+    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="91">
-  <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>K-beauty accessories</t>
-  </si>
-  <si>
-    <t>Scalp massage brush</t>
-  </si>
-  <si>
-    <t>Silicone facial cleansing pad</t>
-  </si>
-  <si>
-    <t>Makeup puff</t>
-  </si>
-  <si>
-    <t>Cosmetic spatula</t>
-  </si>
-  <si>
-    <t>Cosmetic organizer</t>
-  </si>
-  <si>
-    <t>Travel cosmetic bottle</t>
-  </si>
-  <si>
-    <t>Ice face roller</t>
-  </si>
-  <si>
-    <t>Reusable silicone mask cover</t>
-  </si>
-  <si>
-    <t>Blackhead remover tool kit</t>
-  </si>
-  <si>
-    <t>Mini skincare fridge organizer</t>
-  </si>
-  <si>
-    <t>Hair &amp; scalp care tools</t>
-  </si>
-  <si>
-    <t>Shower scalp brush</t>
-  </si>
-  <si>
-    <t>Hair towel</t>
-  </si>
-  <si>
-    <t>Compact comb</t>
-  </si>
-  <si>
-    <t>Brush holder</t>
-  </si>
-  <si>
-    <t>Heatless hair curler</t>
-  </si>
-  <si>
-    <t>Hair section clips</t>
-  </si>
-  <si>
-    <t>Portable detangling brush</t>
-  </si>
-  <si>
-    <t>Scalp oil applicator bottle</t>
-  </si>
-  <si>
-    <t>Korean lifestyle small goods</t>
-  </si>
-  <si>
-    <t>Desk organizer</t>
-  </si>
-  <si>
-    <t>Cute stationery</t>
-  </si>
-  <si>
-    <t>Travel pouch</t>
-  </si>
-  <si>
-    <t>Kitchen small tool</t>
-  </si>
-  <si>
-    <t>Storage case</t>
-  </si>
-  <si>
-    <t>Cable organizer</t>
-  </si>
-  <si>
-    <t>Mini trash bin for desk</t>
-  </si>
-  <si>
-    <t>Reusable shopping bag</t>
-  </si>
-  <si>
-    <t>Foldable laundry basket</t>
-  </si>
-  <si>
-    <t>Refrigerator storage box</t>
-  </si>
-  <si>
-    <t>Korean desk &amp; study accessories</t>
-  </si>
-  <si>
-    <t>Laptop stand</t>
-  </si>
-  <si>
-    <t>Keyboard cleaning gel</t>
-  </si>
-  <si>
-    <t>Monitor memo board</t>
-  </si>
-  <si>
-    <t>Aesthetic mouse pad</t>
-  </si>
-  <si>
-    <t>Tablet stand</t>
-  </si>
-  <si>
-    <t>Korean travel accessories</t>
-  </si>
-  <si>
-    <t>Compression packing cubes</t>
-  </si>
-  <si>
-    <t>Passport holder</t>
-  </si>
-  <si>
-    <t>Portable jewelry case</t>
-  </si>
-  <si>
-    <t>Mini refill perfume bottle</t>
-  </si>
-  <si>
-    <t>Luggage shoe bag</t>
-  </si>
-  <si>
-    <t>Korean pet accessories</t>
-  </si>
-  <si>
-    <t>Pet grooming glove</t>
-  </si>
-  <si>
-    <t>Portable pet water bottle</t>
-  </si>
-  <si>
-    <t>Pet food storage container</t>
-  </si>
-  <si>
-    <t>Silicone pet bath brush</t>
-  </si>
-  <si>
-    <t>Pet hair remover roller</t>
-  </si>
-  <si>
-    <t>product_name</t>
-  </si>
-  <si>
-    <t>order_this_month</t>
-  </si>
-  <si>
-    <t>order_last_month</t>
-  </si>
-  <si>
-    <t>search_this_month</t>
-  </si>
-  <si>
-    <t>search_last_month</t>
-  </si>
-  <si>
-    <t>review_this_month</t>
-  </si>
-  <si>
-    <t>review_last_month</t>
-  </si>
-  <si>
-    <t>selling_price</t>
-  </si>
-  <si>
-    <t>product_cost</t>
-  </si>
-  <si>
-    <t>shipping_cost</t>
-  </si>
-  <si>
-    <t>platform_fees</t>
-  </si>
-  <si>
-    <t>number_of_competitors</t>
-  </si>
-  <si>
-    <t>avg_top_five_competitor_reviews</t>
-  </si>
-  <si>
-    <t>avg_margin</t>
-  </si>
-  <si>
-    <t>avg_selling_price</t>
-  </si>
-  <si>
-    <t>delivery_time</t>
-  </si>
-  <si>
-    <t>weight</t>
-  </si>
-  <si>
-    <t>fragility</t>
-  </si>
-  <si>
-    <t>supplier_rating</t>
-  </si>
-  <si>
-    <t>moq</t>
-  </si>
-  <si>
-    <t>response_rate</t>
-  </si>
-  <si>
-    <t>supplier_completed_orders</t>
-  </si>
-  <si>
-    <t>supplier_max_orders</t>
-  </si>
-  <si>
-    <t>current_tiktok_trend_score</t>
-  </si>
-  <si>
-    <t>last_month_tiktok_trend_score</t>
-  </si>
-  <si>
-    <t>number_of_creators</t>
-  </si>
-  <si>
-    <t>size</t>
-  </si>
-  <si>
-    <t>advertising_costs</t>
-  </si>
-  <si>
-    <t>product_category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">selling price </t>
-  </si>
-  <si>
-    <t>avg in usd</t>
-  </si>
-  <si>
-    <t>median in usd</t>
-  </si>
-  <si>
-    <t>avg in KRW</t>
-  </si>
-  <si>
-    <t>median in KRW</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KRW to USD </t>
-  </si>
-  <si>
-    <t>Data Source</t>
-  </si>
-  <si>
-    <t>Shopee</t>
-  </si>
-  <si>
-    <t>https://chinaggook.domeggook.com/home/product/list.php?ss=1688&amp;sk=name&amp;sv=Scalp%20massage%20brush&amp;img=#n</t>
-  </si>
-  <si>
-    <t>shopee fee rate</t>
-  </si>
-  <si>
-    <t>https://shopee.kr/edu/article/10624</t>
-  </si>
-  <si>
-    <t xml:space="preserve">advertising costs rate </t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="79">
+  <si>
+    <t xml:space="preserve">id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product_name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product_category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">selling_price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">product_cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shipping_cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">platform_fees</t>
+  </si>
+  <si>
+    <t xml:space="preserve">advertising_costs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">order_this_month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">order_last_month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">search_this_month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">search_last_month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">review_this_month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">review_last_month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">number_of_competitors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avg_top_five_competitor_reviews</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avg_margin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">avg_selling_price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">delivery_time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">weight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fragility</t>
+  </si>
+  <si>
+    <t xml:space="preserve">supplier_rating</t>
+  </si>
+  <si>
+    <t xml:space="preserve">moq</t>
+  </si>
+  <si>
+    <t xml:space="preserve">response_rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">supplier_completed_orders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">supplier_max_orders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">current_tiktok_trend_score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">last_month_tiktok_trend_score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">number_of_creators</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scalp massage brush</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K-beauty accessories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Silicone facial cleansing pad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Makeup puff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosmetic spatula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cosmetic organizer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travel cosmetic bottle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ice face roller</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reusable silicone mask cover</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blackhead remover tool kit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mini skincare fridge organizer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shower scalp brush</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hair &amp; scalp care tools</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hair towel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compact comb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brush holder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heatless hair curler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hair section clips</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portable detangling brush</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scalp oil applicator bottle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desk organizer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Korean lifestyle small goods</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cute stationery</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travel pouch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kitchen small tool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Storage case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cable organizer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mini trash bin for desk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reusable shopping bag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foldable laundry basket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Refrigerator storage box</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Laptop stand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Korean desk &amp; study accessories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keyboard cleaning gel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monitor memo board</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aesthetic mouse pad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tablet stand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compression packing cubes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Korean travel accessories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Passport holder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portable jewelry case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mini refill perfume bottle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luggage shoe bag</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pet grooming glove</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Korean pet accessories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portable pet water bottle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pet food storage container</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Silicone pet bath brush</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pet hair remover roller</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="General"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -322,208 +300,159 @@
     </fill>
   </fills>
   <borders count="2">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thème Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="44546a"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="e7e6e6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="5b9bd5"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="ed7d31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="a5a5a5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="ffc000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4472c4"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="70ad47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0563c1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="954f72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme>
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
                 <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
                 <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
                 <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
                 <a:lumMod val="102000"/>
                 <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
                 <a:lumMod val="100000"/>
                 <a:shade val="100000"/>
               </a:schemeClr>
@@ -531,33 +460,24 @@
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
                 <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
@@ -570,13 +490,7 @@
           <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
+          <a:effectLst/>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -586,15 +500,13 @@
         <a:solidFill>
           <a:schemeClr val="phClr">
             <a:tint val="95000"/>
-            <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
-                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
               </a:schemeClr>
@@ -602,7 +514,6 @@
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
-                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
               </a:schemeClr>
@@ -610,135 +521,135 @@
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="63000"/>
-                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:AD44"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="10.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.5546875" bestFit="1" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="27.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="13.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10.16"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>78</v>
+        <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>57</v>
+        <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>58</v>
+        <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>59</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>60</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>77</v>
+        <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>51</v>
+        <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>52</v>
+        <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>53</v>
+        <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>54</v>
+        <v>11</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>56</v>
+        <v>13</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>61</v>
+        <v>14</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>62</v>
+        <v>15</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>63</v>
+        <v>16</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>64</v>
+        <v>17</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>65</v>
+        <v>18</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>66</v>
+        <v>19</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>76</v>
+        <v>20</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>67</v>
+        <v>21</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>68</v>
+        <v>22</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>69</v>
+        <v>23</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>70</v>
+        <v>24</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>71</v>
+        <v>25</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>73</v>
+        <v>27</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>74</v>
+        <v>28</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -768,15 +679,15 @@
       <c r="AC2" s="1"/>
       <c r="AD2" s="1"/>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -806,15 +717,15 @@
       <c r="AC3" s="1"/>
       <c r="AD3" s="1"/>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -844,15 +755,15 @@
       <c r="AC4" s="1"/>
       <c r="AD4" s="1"/>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -882,15 +793,15 @@
       <c r="AC5" s="1"/>
       <c r="AD5" s="1"/>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -920,15 +831,15 @@
       <c r="AC6" s="1"/>
       <c r="AD6" s="1"/>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -958,15 +869,15 @@
       <c r="AC7" s="1"/>
       <c r="AD7" s="1"/>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A8" s="1">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
@@ -996,15 +907,15 @@
       <c r="AC8" s="1"/>
       <c r="AD8" s="1"/>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -1034,15 +945,15 @@
       <c r="AC9" s="1"/>
       <c r="AD9" s="1"/>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -1072,15 +983,15 @@
       <c r="AC10" s="1"/>
       <c r="AD10" s="1"/>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A11" s="1">
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -1110,15 +1021,15 @@
       <c r="AC11" s="1"/>
       <c r="AD11" s="1"/>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A12" s="1">
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -1148,15 +1059,15 @@
       <c r="AC12" s="1"/>
       <c r="AD12" s="1"/>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A13" s="1">
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
@@ -1186,15 +1097,15 @@
       <c r="AC13" s="1"/>
       <c r="AD13" s="1"/>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A14" s="1">
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="n">
         <v>13</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
@@ -1224,15 +1135,15 @@
       <c r="AC14" s="1"/>
       <c r="AD14" s="1"/>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A15" s="1">
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>16</v>
+        <v>45</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
@@ -1262,15 +1173,15 @@
       <c r="AC15" s="1"/>
       <c r="AD15" s="1"/>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A16" s="1">
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="n">
         <v>15</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
@@ -1300,15 +1211,15 @@
       <c r="AC16" s="1"/>
       <c r="AD16" s="1"/>
     </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A17" s="1">
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="n">
         <v>16</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>18</v>
+        <v>47</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
@@ -1338,15 +1249,15 @@
       <c r="AC17" s="1"/>
       <c r="AD17" s="1"/>
     </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A18" s="1">
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="n">
         <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>19</v>
+        <v>48</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
@@ -1376,15 +1287,15 @@
       <c r="AC18" s="1"/>
       <c r="AD18" s="1"/>
     </row>
-    <row r="19" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A19" s="1">
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="n">
         <v>18</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>20</v>
+        <v>49</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
@@ -1414,15 +1325,15 @@
       <c r="AC19" s="1"/>
       <c r="AD19" s="1"/>
     </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A20" s="1">
+    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="n">
         <v>19</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
@@ -1452,15 +1363,15 @@
       <c r="AC20" s="1"/>
       <c r="AD20" s="1"/>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A21" s="1">
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="n">
         <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>23</v>
+        <v>52</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
@@ -1490,15 +1401,15 @@
       <c r="AC21" s="1"/>
       <c r="AD21" s="1"/>
     </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A22" s="1">
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="n">
         <v>21</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
@@ -1528,15 +1439,15 @@
       <c r="AC22" s="1"/>
       <c r="AD22" s="1"/>
     </row>
-    <row r="23" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A23" s="1">
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="n">
         <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
@@ -1566,15 +1477,15 @@
       <c r="AC23" s="1"/>
       <c r="AD23" s="1"/>
     </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A24" s="1">
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="n">
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
@@ -1604,15 +1515,15 @@
       <c r="AC24" s="1"/>
       <c r="AD24" s="1"/>
     </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A25" s="1">
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="n">
         <v>24</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>27</v>
+        <v>56</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
@@ -1642,15 +1553,15 @@
       <c r="AC25" s="1"/>
       <c r="AD25" s="1"/>
     </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A26" s="1">
+    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="n">
         <v>25</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
@@ -1680,15 +1591,15 @@
       <c r="AC26" s="1"/>
       <c r="AD26" s="1"/>
     </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A27" s="1">
+    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="n">
         <v>26</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>29</v>
+        <v>58</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
@@ -1718,15 +1629,15 @@
       <c r="AC27" s="1"/>
       <c r="AD27" s="1"/>
     </row>
-    <row r="28" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A28" s="1">
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="n">
         <v>27</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>30</v>
+        <v>59</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
@@ -1756,15 +1667,15 @@
       <c r="AC28" s="1"/>
       <c r="AD28" s="1"/>
     </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A29" s="1">
+    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="n">
         <v>28</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>31</v>
+        <v>60</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
@@ -1794,15 +1705,15 @@
       <c r="AC29" s="1"/>
       <c r="AD29" s="1"/>
     </row>
-    <row r="30" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A30" s="1">
+    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="n">
         <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>32</v>
+        <v>62</v>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
@@ -1832,15 +1743,15 @@
       <c r="AC30" s="1"/>
       <c r="AD30" s="1"/>
     </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A31" s="1">
+    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="n">
         <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>32</v>
+        <v>62</v>
       </c>
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
@@ -1870,15 +1781,15 @@
       <c r="AC31" s="1"/>
       <c r="AD31" s="1"/>
     </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A32" s="1">
+    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="n">
         <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>32</v>
+        <v>62</v>
       </c>
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
@@ -1908,15 +1819,15 @@
       <c r="AC32" s="1"/>
       <c r="AD32" s="1"/>
     </row>
-    <row r="33" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A33" s="1">
+    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="n">
         <v>32</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>32</v>
+        <v>62</v>
       </c>
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
@@ -1946,15 +1857,15 @@
       <c r="AC33" s="1"/>
       <c r="AD33" s="1"/>
     </row>
-    <row r="34" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A34" s="1">
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="n">
         <v>33</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>37</v>
+        <v>66</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>32</v>
+        <v>62</v>
       </c>
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
@@ -1984,15 +1895,15 @@
       <c r="AC34" s="1"/>
       <c r="AD34" s="1"/>
     </row>
-    <row r="35" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A35" s="1">
+    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="n">
         <v>34</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
@@ -2022,15 +1933,15 @@
       <c r="AC35" s="1"/>
       <c r="AD35" s="1"/>
     </row>
-    <row r="36" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A36" s="1">
+    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="n">
         <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>40</v>
+        <v>69</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
@@ -2060,15 +1971,15 @@
       <c r="AC36" s="1"/>
       <c r="AD36" s="1"/>
     </row>
-    <row r="37" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A37" s="1">
+    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="n">
         <v>36</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>41</v>
+        <v>70</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
@@ -2098,15 +2009,15 @@
       <c r="AC37" s="1"/>
       <c r="AD37" s="1"/>
     </row>
-    <row r="38" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A38" s="1">
+    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="n">
         <v>37</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>42</v>
+        <v>71</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
@@ -2136,15 +2047,15 @@
       <c r="AC38" s="1"/>
       <c r="AD38" s="1"/>
     </row>
-    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A39" s="1">
+    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="n">
         <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>43</v>
+        <v>72</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
@@ -2174,15 +2085,15 @@
       <c r="AC39" s="1"/>
       <c r="AD39" s="1"/>
     </row>
-    <row r="40" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A40" s="1">
+    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="n">
         <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>45</v>
+        <v>73</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
@@ -2212,15 +2123,15 @@
       <c r="AC40" s="1"/>
       <c r="AD40" s="1"/>
     </row>
-    <row r="41" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A41" s="1">
+    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="n">
         <v>40</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="D41" s="1"/>
       <c r="E41" s="1"/>
@@ -2250,15 +2161,15 @@
       <c r="AC41" s="1"/>
       <c r="AD41" s="1"/>
     </row>
-    <row r="42" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A42" s="1">
+    <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="n">
         <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>47</v>
+        <v>76</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="D42" s="1"/>
       <c r="E42" s="1"/>
@@ -2288,15 +2199,15 @@
       <c r="AC42" s="1"/>
       <c r="AD42" s="1"/>
     </row>
-    <row r="43" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A43" s="1">
+    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="n">
         <v>42</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>48</v>
+        <v>77</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="D43" s="1"/>
       <c r="E43" s="1"/>
@@ -2326,15 +2237,15 @@
       <c r="AC43" s="1"/>
       <c r="AD43" s="1"/>
     </row>
-    <row r="44" spans="1:30" x14ac:dyDescent="0.3">
-      <c r="A44" s="1">
+    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="n">
         <v>43</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>49</v>
+        <v>78</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
@@ -2365,294 +2276,35 @@
       <c r="AD44" s="1"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB25"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultColWidth="10.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="15.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16.67"/>
   </cols>
-  <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="B1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="B2">
-        <v>200</v>
-      </c>
-      <c r="C2">
-        <v>4767</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="B3">
-        <v>128</v>
-      </c>
-      <c r="C3">
-        <v>1646</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="B4">
-        <v>205</v>
-      </c>
-      <c r="C4">
-        <v>3183</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="B5">
-        <v>329</v>
-      </c>
-      <c r="C5">
-        <v>5844</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="B6">
-        <v>255</v>
-      </c>
-      <c r="C6">
-        <v>5029</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="B7">
-        <v>300</v>
-      </c>
-      <c r="C7">
-        <v>15223</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="B8">
-        <v>300</v>
-      </c>
-      <c r="C8">
-        <v>2691</v>
-      </c>
-    </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="B9">
-        <v>100</v>
-      </c>
-      <c r="C9">
-        <v>7228</v>
-      </c>
-    </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="B10">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="B11">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>82</v>
-      </c>
-      <c r="C12">
-        <f>AVERAGEA(C2:C11)</f>
-        <v>5701.375</v>
-      </c>
-      <c r="D12">
-        <v>14000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>83</v>
-      </c>
-      <c r="C13">
-        <f xml:space="preserve"> MEDIAN(C2:C11)</f>
-        <v>4898</v>
-      </c>
-      <c r="D13">
-        <v>14000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>80</v>
-      </c>
-      <c r="B14">
-        <f>AVERAGEA(B2:B11)</f>
-        <v>243.7</v>
-      </c>
-      <c r="C14">
-        <f>0.00066*C12</f>
-        <v>3.7629074999999998</v>
-      </c>
-      <c r="D14">
-        <f>B18*D12</f>
-        <v>9.24</v>
-      </c>
-      <c r="E14">
-        <f>B23*B14</f>
-        <v>30.09695</v>
-      </c>
-      <c r="F14">
-        <f>B25*B14</f>
-        <v>36.555</v>
-      </c>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>81</v>
-      </c>
-      <c r="B15">
-        <f xml:space="preserve"> MEDIAN(B2:B11)</f>
-        <v>230</v>
-      </c>
-      <c r="C15">
-        <f>0.00066*C13</f>
-        <v>3.2326799999999998</v>
-      </c>
-      <c r="D15">
-        <f>D13*B18</f>
-        <v>9.24</v>
-      </c>
-      <c r="E15">
-        <f>B23*B15</f>
-        <v>28.405000000000001</v>
-      </c>
-      <c r="F15">
-        <f>B25*B15</f>
-        <v>34.5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>84</v>
-      </c>
-      <c r="B18">
-        <v>6.6E-4</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>85</v>
-      </c>
-      <c r="B20" t="s">
-        <v>86</v>
-      </c>
-      <c r="C20" t="s">
-        <v>87</v>
-      </c>
-      <c r="D20" t="s">
-        <v>87</v>
-      </c>
-      <c r="E20" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>88</v>
-      </c>
-      <c r="B23">
-        <v>0.1235</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>90</v>
-      </c>
-      <c r="B25">
-        <v>0.15</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <sheetData/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>